<commit_message>
Correcciones criticas: V2 retirado, criterio 95 %, sin hora de muestreo, citas AT 577, codigo CODESYS limpio
</commit_message>
<xml_diff>
--- a/python/resultados/financiero/flujos_financieros.xlsx
+++ b/python/resultados/financiero/flujos_financieros.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luisi\Downloads\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DB3840A-8F32-432E-84BC-FC5E20B7B430}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Supuestos" sheetId="1" r:id="rId1"/>
@@ -14,7 +20,23 @@
     <sheet name="Operacion_P1C75" sheetId="5" r:id="rId5"/>
     <sheet name="Costo_academico" sheetId="6" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -126,7 +148,7 @@
     <t>Muestreo de humedad al final del lote [h]</t>
   </si>
   <si>
-    <t>Varias muestras para decidir el fin</t>
+    <t>No se cuenta como ahorro: el muestreo final sigue siendo manual</t>
   </si>
   <si>
     <t>Recargo nocturno</t>
@@ -315,13 +337,13 @@
     <t>Alternativa A — escenario Central</t>
   </si>
   <si>
-    <t>2.0 años / 2.5 años</t>
+    <t>2.2 años / 2.8 años</t>
   </si>
   <si>
     <t>Alternativa A — escenario Favorable</t>
   </si>
   <si>
-    <t>1.1 años / 1.2 años</t>
+    <t>1.1 años / 1.3 años</t>
   </si>
   <si>
     <t>Alternativa B — escenario Conservador</t>
@@ -330,13 +352,13 @@
     <t>Alternativa B — escenario Central</t>
   </si>
   <si>
-    <t>1.6 años / 1.9 años</t>
+    <t>1.8 años / 2.1 años</t>
   </si>
   <si>
     <t>Alternativa B — escenario Favorable</t>
   </si>
   <si>
-    <t>0.9 años / 0.9 años</t>
+    <t>0.9 años / 1.0 años</t>
   </si>
   <si>
     <t>Grupo</t>
@@ -597,12 +619,11 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="#,##0"/>
-    <numFmt numFmtId="165" formatCode="0.0%"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -627,7 +648,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -635,17 +656,56 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -653,13 +713,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -697,7 +765,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -731,6 +799,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -765,9 +834,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -940,584 +1010,585 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H39"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="46.7109375" customWidth="1"/>
-    <col min="2" max="2" width="16.7109375" customWidth="1"/>
-    <col min="3" max="3" width="11.7109375" customWidth="1"/>
-    <col min="4" max="4" width="80.7109375" customWidth="1"/>
+    <col min="1" max="1" width="46.6640625" customWidth="1"/>
+    <col min="2" max="2" width="16.6640625" customWidth="1"/>
+    <col min="3" max="3" width="11.6640625" customWidth="1"/>
+    <col min="4" max="4" width="110.88671875" customWidth="1"/>
+    <col min="5" max="9" width="15.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
-      <c r="A2" t="s">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="7">
         <v>14333890</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="6" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
-      <c r="A3" t="s">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="7">
         <v>16828260</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="6" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
-      <c r="A4" t="s">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="7">
         <v>2526946</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="6" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
-      <c r="A5" t="s">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5" s="7">
         <v>11806944</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="6" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
-      <c r="A6" t="s">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6" s="7">
         <v>7352547</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="6" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
-      <c r="A7" t="s">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="2">
+      <c r="B7" s="7">
         <v>9475713</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="6" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
-      <c r="A8" t="s">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="6" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
-      <c r="A9" t="s">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B9" s="2">
+      <c r="B9" s="7">
         <v>468.88</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="6" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
-      <c r="A10" t="s">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B10" s="2">
-        <v>4266.6</v>
-      </c>
-      <c r="C10" t="s">
+      <c r="B10" s="7">
+        <v>4266.6000000000004</v>
+      </c>
+      <c r="C10" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="6" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:4">
-      <c r="A11" t="s">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B11" s="2">
+      <c r="B11" s="7">
         <v>2740717</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="6" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:4">
-      <c r="A12" t="s">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="6">
         <v>0</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="6" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="13" spans="1:4">
-      <c r="A13" t="s">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B13" s="2">
+      <c r="B13" s="7">
         <v>2400000</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="6" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="14" spans="1:4">
-      <c r="A14" t="s">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="6">
         <v>20</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="6" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="15" spans="1:4">
-      <c r="A15" t="s">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="B15">
-        <v>1</v>
-      </c>
-      <c r="C15" t="s">
+      <c r="B15" s="8">
+        <v>0</v>
+      </c>
+      <c r="C15" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="6" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="16" spans="1:4">
-      <c r="A16" t="s">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B16" s="3">
+      <c r="B16" s="8">
         <v>0.35</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="17" spans="1:4">
-      <c r="A17" t="s">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="B17" s="2">
-        <v>1144.3472</v>
-      </c>
-      <c r="C17" t="s">
+      <c r="B17" s="7">
+        <v>1144.3471999999999</v>
+      </c>
+      <c r="C17" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="6" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="18" spans="1:4">
-      <c r="A18" t="s">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="B18" s="2">
-        <v>953.6227</v>
-      </c>
-      <c r="C18" t="s">
+      <c r="B18" s="7">
+        <v>953.62270000000001</v>
+      </c>
+      <c r="C18" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D18" s="6" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="19" spans="1:4">
-      <c r="A19" t="s">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="B19" s="2">
+      <c r="B19" s="7">
         <v>1750905</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D19" s="6" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="20" spans="1:4">
-      <c r="A20" t="s">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="B20">
+      <c r="B20" s="6">
         <v>1.52</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D20" s="6" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="21" spans="1:4">
-      <c r="A21" t="s">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="B21" s="2">
+      <c r="B21" s="7">
         <v>210</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D21" s="6" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="22" spans="1:4">
-      <c r="A22" t="s">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="B22" s="2">
+      <c r="B22" s="7">
         <v>12673.21714285714</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D22" s="6" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="23" spans="1:4">
-      <c r="A23" t="s">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="B23" s="2">
+      <c r="B23" s="7">
         <v>2235000</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D23" s="6" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="24" spans="1:4">
-      <c r="A24" t="s">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="B24" s="3">
+      <c r="B24" s="8">
         <v>0.1895</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C24" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D24" s="6" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="25" spans="1:4">
-      <c r="A25" t="s">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B25" s="3">
-        <v>0.062</v>
-      </c>
-      <c r="C25" t="s">
+      <c r="B25" s="8">
+        <v>6.2E-2</v>
+      </c>
+      <c r="C25" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D25" t="s">
+      <c r="D25" s="6" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="26" spans="1:4">
-      <c r="A26" t="s">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="B26" s="3">
-        <v>0.1200564971751412</v>
-      </c>
-      <c r="C26" t="s">
+      <c r="B26" s="8">
+        <v>0.12005649717514121</v>
+      </c>
+      <c r="C26" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D26" t="s">
+      <c r="D26" s="6" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="27" spans="1:4">
-      <c r="A27" t="s">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A27" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="B27">
+      <c r="B27" s="6">
         <v>5</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C27" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="D27" t="s">
+      <c r="D27" s="6" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="28" spans="1:4">
-      <c r="A28" t="s">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A28" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="B28" s="2">
+      <c r="B28" s="7">
         <v>140.5580888888887</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C28" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="D28" t="s">
+      <c r="D28" s="6" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="29" spans="1:4">
-      <c r="A29" t="s">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A29" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="B29" s="2">
-        <v>117.5597253472205</v>
-      </c>
-      <c r="C29" t="s">
+      <c r="B29" s="7">
+        <v>117.55972534722051</v>
+      </c>
+      <c r="C29" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="D29" t="s">
+      <c r="D29" s="6" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="30" spans="1:4">
-      <c r="A30" t="s">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A30" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="B30">
-        <v>2.754547582181807</v>
-      </c>
-      <c r="C30" t="s">
+      <c r="B30" s="6">
+        <v>2.7545475821818068</v>
+      </c>
+      <c r="C30" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="D30" t="s">
+      <c r="D30" s="6" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="31" spans="1:4">
-      <c r="A31" t="s">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A31" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B31" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C31" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="D31" t="s">
+      <c r="D31" s="6" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="32" spans="1:4">
-      <c r="A32" t="s">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A32" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="B32" t="s">
+      <c r="B32" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="C32" t="s">
+      <c r="C32" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="D32" t="s">
+      <c r="D32" s="6" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="33" spans="1:8">
-      <c r="A33" t="s">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A33" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="B33">
+      <c r="B33" s="6">
         <v>0</v>
       </c>
-      <c r="C33" t="s">
+      <c r="C33" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="D33" t="s">
+      <c r="D33" s="6" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="35" spans="1:8">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="36" spans="1:8">
-      <c r="A36" s="1" t="s">
+    <row r="36" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A36" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="B36" s="1" t="s">
+      <c r="B36" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="C36" s="1" t="s">
+      <c r="C36" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="D36" s="1" t="s">
+      <c r="D36" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="E36" s="1" t="s">
+      <c r="E36" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="F36" s="1" t="s">
+      <c r="F36" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="G36" s="1" t="s">
+      <c r="G36" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="H36" s="1" t="s">
+      <c r="H36" s="9" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="37" spans="1:8">
-      <c r="A37" t="s">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A37" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="B37">
+      <c r="B37" s="6">
         <v>20</v>
       </c>
-      <c r="C37" s="3">
+      <c r="C37" s="8">
         <v>0.16</v>
       </c>
-      <c r="D37">
+      <c r="D37" s="6">
         <v>5</v>
       </c>
-      <c r="E37">
+      <c r="E37" s="6">
         <v>0</v>
       </c>
-      <c r="F37">
+      <c r="F37" s="6">
         <v>4</v>
       </c>
-      <c r="G37" s="3">
+      <c r="G37" s="8">
         <v>0.04</v>
       </c>
-      <c r="H37" s="3">
+      <c r="H37" s="8">
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:8">
-      <c r="A38" t="s">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A38" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="B38">
+      <c r="B38" s="6">
         <v>40</v>
       </c>
-      <c r="C38" s="3">
-        <v>0.1200564971751412</v>
-      </c>
-      <c r="D38">
+      <c r="C38" s="8">
+        <v>0.12005649717514121</v>
+      </c>
+      <c r="D38" s="6">
         <v>10</v>
       </c>
-      <c r="E38">
+      <c r="E38" s="6">
         <v>0.5</v>
       </c>
-      <c r="F38">
+      <c r="F38" s="6">
         <v>8</v>
       </c>
-      <c r="G38" s="3">
+      <c r="G38" s="8">
         <v>0.03</v>
       </c>
-      <c r="H38" s="3">
+      <c r="H38" s="8">
         <v>0.2</v>
       </c>
     </row>
-    <row r="39" spans="1:8">
-      <c r="A39" t="s">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A39" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="B39">
+      <c r="B39" s="6">
         <v>60</v>
       </c>
-      <c r="C39" s="3">
+      <c r="C39" s="8">
         <v>0.08</v>
       </c>
-      <c r="D39">
+      <c r="D39" s="6">
         <v>15</v>
       </c>
-      <c r="E39">
+      <c r="E39" s="6">
         <v>1</v>
       </c>
-      <c r="F39">
+      <c r="F39" s="6">
         <v>12</v>
       </c>
-      <c r="G39" s="3">
+      <c r="G39" s="8">
         <v>0.02</v>
       </c>
-      <c r="H39" s="3">
+      <c r="H39" s="8">
         <v>0.4</v>
       </c>
     </row>
@@ -1527,967 +1598,1147 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G71"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="34.7109375" customWidth="1"/>
-    <col min="2" max="8" width="14.7109375" customWidth="1"/>
+    <col min="1" max="1" width="34.6640625" customWidth="1"/>
+    <col min="2" max="8" width="14.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="B2" s="1">
+      <c r="B2" s="5">
         <v>0</v>
       </c>
-      <c r="C2" s="1">
+      <c r="C2" s="5">
         <v>1</v>
       </c>
-      <c r="D2" s="1">
+      <c r="D2" s="5">
         <v>2</v>
       </c>
-      <c r="E2" s="1">
+      <c r="E2" s="5">
         <v>3</v>
       </c>
-      <c r="F2" s="1">
+      <c r="F2" s="5">
         <v>4</v>
       </c>
-      <c r="G2" s="1">
+      <c r="G2" s="5">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
-      <c r="A3" t="s">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="7">
         <v>-11806944</v>
       </c>
-      <c r="C3" s="2">
-        <v>1702606</v>
-      </c>
-      <c r="D3" s="2">
-        <v>1702606</v>
-      </c>
-      <c r="E3" s="2">
-        <v>1702606</v>
-      </c>
-      <c r="F3" s="2">
-        <v>1702606</v>
-      </c>
-      <c r="G3" s="2">
-        <v>1702606</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" t="s">
+      <c r="C3" s="7">
+        <v>1449142</v>
+      </c>
+      <c r="D3" s="7">
+        <v>1449142</v>
+      </c>
+      <c r="E3" s="7">
+        <v>1449142</v>
+      </c>
+      <c r="F3" s="7">
+        <v>1449142</v>
+      </c>
+      <c r="G3" s="7">
+        <v>1449142</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="8">
         <v>0.16</v>
       </c>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5" t="s">
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5" s="7">
         <f>NPV(B4,C3:G3)+B3</f>
-        <v>-6232110</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6" t="s">
+        <v>-7062027.5461460492</v>
+      </c>
+      <c r="C5" s="6"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="8">
         <f>IRR(B3:G3)</f>
-        <v>-0.09998144505325796</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
-      <c r="A7" t="s">
+        <v>-0.14342348792062098</v>
+      </c>
+      <c r="C6" s="6"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
+      <c r="F6" s="6"/>
+      <c r="G6" s="6"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="B7" s="2">
+      <c r="B7" s="7">
         <f>B3</f>
         <v>-11806944</v>
       </c>
-      <c r="C7" s="2">
+      <c r="C7" s="7">
         <f>B7+C3</f>
-        <v>-10104338</v>
-      </c>
-      <c r="D7" s="2">
+        <v>-10357802</v>
+      </c>
+      <c r="D7" s="7">
         <f>C7+D3</f>
-        <v>-8401731</v>
-      </c>
-      <c r="E7" s="2">
+        <v>-8908660</v>
+      </c>
+      <c r="E7" s="7">
         <f>D7+E3</f>
-        <v>-6699125</v>
-      </c>
-      <c r="F7" s="2">
+        <v>-7459518</v>
+      </c>
+      <c r="F7" s="7">
         <f>E7+F3</f>
-        <v>-4996518</v>
-      </c>
-      <c r="G7" s="2">
+        <v>-6010376</v>
+      </c>
+      <c r="G7" s="7">
         <f>F7+G3</f>
-        <v>-3293912</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7">
-      <c r="A8" t="s">
+        <v>-4561234</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="B8" s="2">
+      <c r="B8" s="7">
         <f>B3</f>
         <v>-11806944</v>
       </c>
-      <c r="C8" s="2">
+      <c r="C8" s="7">
         <f>B8+C3/(1+B4)^1</f>
-        <v>-10339180</v>
-      </c>
-      <c r="D8" s="2">
+        <v>-10557683.655172413</v>
+      </c>
+      <c r="D8" s="7">
         <f>C8+D3/(1+B4)^2</f>
-        <v>-9073866</v>
-      </c>
-      <c r="E8" s="2">
+        <v>-9480735.0820451844</v>
+      </c>
+      <c r="E8" s="7">
         <f>D8+E3/(1+B4)^3</f>
-        <v>-7983078</v>
-      </c>
-      <c r="F8" s="2">
+        <v>-8552331.1396941245</v>
+      </c>
+      <c r="F8" s="7">
         <f>E8+F3/(1+B4)^4</f>
-        <v>-7042744</v>
-      </c>
-      <c r="G8" s="2">
+        <v>-7751982.9135294175</v>
+      </c>
+      <c r="G8" s="7">
         <f>F8+G3/(1+B4)^5</f>
-        <v>-6232110</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7">
-      <c r="A9" t="s">
+        <v>-7062027.5461460492</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="6" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="10" spans="1:7">
-      <c r="A10" t="s">
+      <c r="C9" s="6"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="6"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B10" s="2">
-        <v>103944</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7">
-      <c r="A11" t="s">
+      <c r="B10" s="7">
+        <v>91271</v>
+      </c>
+      <c r="C10" s="6"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="6"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="B11" s="2">
+      <c r="B11" s="7">
         <v>199111</v>
       </c>
-    </row>
-    <row r="13" spans="1:7">
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="6"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="14" spans="1:7">
-      <c r="A14" s="1" t="s">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="B14" s="1">
+      <c r="B14" s="5">
         <v>0</v>
       </c>
-      <c r="C14" s="1">
+      <c r="C14" s="5">
         <v>1</v>
       </c>
-      <c r="D14" s="1">
+      <c r="D14" s="5">
         <v>2</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="5">
         <v>3</v>
       </c>
-      <c r="F14" s="1">
+      <c r="F14" s="5">
         <v>4</v>
       </c>
-      <c r="G14" s="1">
+      <c r="G14" s="5">
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:7">
-      <c r="A15" t="s">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="B15" s="2">
+      <c r="B15" s="7">
         <v>-11806944</v>
       </c>
-      <c r="C15" s="2">
-        <v>5803230</v>
-      </c>
-      <c r="D15" s="2">
-        <v>5803230</v>
-      </c>
-      <c r="E15" s="2">
-        <v>5803230</v>
-      </c>
-      <c r="F15" s="2">
-        <v>5803230</v>
-      </c>
-      <c r="G15" s="2">
-        <v>7684619</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7">
-      <c r="A16" t="s">
+      <c r="C15" s="7">
+        <v>5296301</v>
+      </c>
+      <c r="D15" s="7">
+        <v>5296301</v>
+      </c>
+      <c r="E15" s="7">
+        <v>5296301</v>
+      </c>
+      <c r="F15" s="7">
+        <v>5296301</v>
+      </c>
+      <c r="G15" s="7">
+        <v>7177690</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="B16" s="3">
-        <v>0.1200564971751412</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7">
-      <c r="A17" t="s">
+      <c r="B16" s="8">
+        <v>0.12005649717514121</v>
+      </c>
+      <c r="C16" s="6"/>
+      <c r="D16" s="6"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="6"/>
+      <c r="G16" s="6"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A17" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="B17" s="2">
+      <c r="B17" s="7">
         <f>NPV(B16,C15:G15)+B15</f>
-        <v>10176754</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7">
-      <c r="A18" t="s">
+        <v>8349645.395731546</v>
+      </c>
+      <c r="C17" s="6"/>
+      <c r="D17" s="6"/>
+      <c r="E17" s="6"/>
+      <c r="F17" s="6"/>
+      <c r="G17" s="6"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A18" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B18" s="3">
+      <c r="B18" s="8">
         <f>IRR(B15:G15)</f>
-        <v>0.4171474325396548</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7">
-      <c r="A19" t="s">
+        <v>0.36678304254416694</v>
+      </c>
+      <c r="C18" s="6"/>
+      <c r="D18" s="6"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
+      <c r="G18" s="6"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="B19" s="2">
+      <c r="B19" s="7">
         <f>B15</f>
         <v>-11806944</v>
       </c>
-      <c r="C19" s="2">
+      <c r="C19" s="7">
         <f>B19+C15</f>
-        <v>-6003714</v>
-      </c>
-      <c r="D19" s="2">
+        <v>-6510643</v>
+      </c>
+      <c r="D19" s="7">
         <f>C19+D15</f>
-        <v>-200484</v>
-      </c>
-      <c r="E19" s="2">
+        <v>-1214342</v>
+      </c>
+      <c r="E19" s="7">
         <f>D19+E15</f>
-        <v>5602745</v>
-      </c>
-      <c r="F19" s="2">
+        <v>4081959</v>
+      </c>
+      <c r="F19" s="7">
         <f>E19+F15</f>
-        <v>11405975</v>
-      </c>
-      <c r="G19" s="2">
+        <v>9378260</v>
+      </c>
+      <c r="G19" s="7">
         <f>F19+G15</f>
-        <v>19090594</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7">
-      <c r="A20" t="s">
+        <v>16555950</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A20" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="B20" s="2">
+      <c r="B20" s="7">
         <f>B15</f>
         <v>-11806944</v>
       </c>
-      <c r="C20" s="2">
+      <c r="C20" s="7">
         <f>B20+C15/(1+B16)^1</f>
-        <v>-6625750</v>
-      </c>
-      <c r="D20" s="2">
+        <v>-7078342.3505674656</v>
+      </c>
+      <c r="D20" s="7">
         <f>C20+D15/(1+B16)^2</f>
-        <v>-1999918</v>
-      </c>
-      <c r="E20" s="2">
+        <v>-2856589.5538483802</v>
+      </c>
+      <c r="E20" s="7">
         <f>D20+E15/(1+B16)^3</f>
-        <v>2130082</v>
-      </c>
-      <c r="F20" s="2">
+        <v>912642.45129299723</v>
+      </c>
+      <c r="F20" s="7">
         <f>E20+F15/(1+B16)^4</f>
-        <v>5817395</v>
-      </c>
-      <c r="G20" s="2">
+        <v>4277858.4155301917</v>
+      </c>
+      <c r="G20" s="7">
         <f>F20+G15/(1+B16)^5</f>
-        <v>10176754</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7">
-      <c r="A21" t="s">
+        <v>8349645.3957315451</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="6" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="22" spans="1:7">
-      <c r="A22" t="s">
+      <c r="C21" s="6"/>
+      <c r="D21" s="6"/>
+      <c r="E21" s="6"/>
+      <c r="F21" s="6"/>
+      <c r="G21" s="6"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A22" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B22" s="2">
-        <v>152136</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7">
-      <c r="A23" t="s">
+      <c r="B22" s="7">
+        <v>139463</v>
+      </c>
+      <c r="C22" s="6"/>
+      <c r="D22" s="6"/>
+      <c r="E22" s="6"/>
+      <c r="F22" s="6"/>
+      <c r="G22" s="6"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A23" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="B23" s="2">
+      <c r="B23" s="7">
         <v>81548</v>
       </c>
-    </row>
-    <row r="25" spans="1:7">
+      <c r="C23" s="6"/>
+      <c r="D23" s="6"/>
+      <c r="E23" s="6"/>
+      <c r="F23" s="6"/>
+      <c r="G23" s="6"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="26" spans="1:7">
-      <c r="A26" s="1" t="s">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A26" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="B26" s="1">
+      <c r="B26" s="5">
         <v>0</v>
       </c>
-      <c r="C26" s="1">
+      <c r="C26" s="5">
         <v>1</v>
       </c>
-      <c r="D26" s="1">
+      <c r="D26" s="5">
         <v>2</v>
       </c>
-      <c r="E26" s="1">
+      <c r="E26" s="5">
         <v>3</v>
       </c>
-      <c r="F26" s="1">
+      <c r="F26" s="5">
         <v>4</v>
       </c>
-      <c r="G26" s="1">
+      <c r="G26" s="5">
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="1:7">
-      <c r="A27" t="s">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A27" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="B27" s="2">
+      <c r="B27" s="7">
         <v>-11806944</v>
       </c>
-      <c r="C27" s="2">
-        <v>11036652</v>
-      </c>
-      <c r="D27" s="2">
-        <v>11036652</v>
-      </c>
-      <c r="E27" s="2">
-        <v>11036652</v>
-      </c>
-      <c r="F27" s="2">
-        <v>11036652</v>
-      </c>
-      <c r="G27" s="2">
-        <v>14799430</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7">
-      <c r="A28" t="s">
+      <c r="C27" s="7">
+        <v>10276259</v>
+      </c>
+      <c r="D27" s="7">
+        <v>10276259</v>
+      </c>
+      <c r="E27" s="7">
+        <v>10276259</v>
+      </c>
+      <c r="F27" s="7">
+        <v>10276259</v>
+      </c>
+      <c r="G27" s="7">
+        <v>14039037</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A28" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="B28" s="3">
+      <c r="B28" s="8">
         <v>0.08</v>
       </c>
-    </row>
-    <row r="29" spans="1:7">
-      <c r="A29" t="s">
+      <c r="C28" s="6"/>
+      <c r="D28" s="6"/>
+      <c r="E28" s="6"/>
+      <c r="F28" s="6"/>
+      <c r="G28" s="6"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A29" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="B29" s="2">
+      <c r="B29" s="7">
         <f>NPV(B28,C27:G27)+B27</f>
-        <v>34820090</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7">
-      <c r="A30" t="s">
+        <v>31784061.933882266</v>
+      </c>
+      <c r="C29" s="6"/>
+      <c r="D29" s="6"/>
+      <c r="E29" s="6"/>
+      <c r="F29" s="6"/>
+      <c r="G29" s="6"/>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A30" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B30" s="3">
+      <c r="B30" s="8">
         <f>IRR(B27:G27)</f>
-        <v>0.9093431097782465</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7">
-      <c r="A31" t="s">
+        <v>0.84196415885167575</v>
+      </c>
+      <c r="C30" s="6"/>
+      <c r="D30" s="6"/>
+      <c r="E30" s="6"/>
+      <c r="F30" s="6"/>
+      <c r="G30" s="6"/>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A31" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="B31" s="2">
+      <c r="B31" s="7">
         <f>B27</f>
         <v>-11806944</v>
       </c>
-      <c r="C31" s="2">
+      <c r="C31" s="7">
         <f>B31+C27</f>
-        <v>-770292</v>
-      </c>
-      <c r="D31" s="2">
+        <v>-1530685</v>
+      </c>
+      <c r="D31" s="7">
         <f>C31+D27</f>
-        <v>10266360</v>
-      </c>
-      <c r="E31" s="2">
+        <v>8745574</v>
+      </c>
+      <c r="E31" s="7">
         <f>D31+E27</f>
-        <v>21303012</v>
-      </c>
-      <c r="F31" s="2">
+        <v>19021833</v>
+      </c>
+      <c r="F31" s="7">
         <f>E31+F27</f>
-        <v>32339664</v>
-      </c>
-      <c r="G31" s="2">
+        <v>29298092</v>
+      </c>
+      <c r="G31" s="7">
         <f>F31+G27</f>
-        <v>47139093</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7">
-      <c r="A32" t="s">
+        <v>43337129</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A32" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="B32" s="2">
+      <c r="B32" s="7">
         <f>B27</f>
         <v>-11806944</v>
       </c>
-      <c r="C32" s="2">
+      <c r="C32" s="7">
         <f>B32+C27/(1+B28)^1</f>
-        <v>-1587822</v>
-      </c>
-      <c r="D32" s="2">
+        <v>-2291889.3703703713</v>
+      </c>
+      <c r="D32" s="7">
         <f>C32+D27/(1+B28)^2</f>
-        <v>7874328</v>
-      </c>
-      <c r="E32" s="2">
+        <v>6518346.3978052102</v>
+      </c>
+      <c r="E32" s="7">
         <f>D32+E27/(1+B28)^3</f>
-        <v>16635579</v>
-      </c>
-      <c r="F32" s="2">
+        <v>14675972.109078897</v>
+      </c>
+      <c r="F32" s="7">
         <f>E32+F27/(1+B28)^4</f>
-        <v>24747847</v>
-      </c>
-      <c r="G32" s="2">
+        <v>22229329.249147125</v>
+      </c>
+      <c r="G32" s="7">
         <f>F32+G27/(1+B28)^5</f>
-        <v>34820090</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7">
-      <c r="A33" t="s">
+        <v>31784061.933882274</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A33" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="B33" t="s">
+      <c r="B33" s="6" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="34" spans="1:7">
-      <c r="A34" t="s">
+      <c r="C33" s="6"/>
+      <c r="D33" s="6"/>
+      <c r="E33" s="6"/>
+      <c r="F33" s="6"/>
+      <c r="G33" s="6"/>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A34" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B34" s="2">
-        <v>187080</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7">
-      <c r="A35" t="s">
+      <c r="B34" s="7">
+        <v>174407</v>
+      </c>
+      <c r="C34" s="6"/>
+      <c r="D34" s="6"/>
+      <c r="E34" s="6"/>
+      <c r="F34" s="6"/>
+      <c r="G34" s="6"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A35" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="B35" s="2">
+      <c r="B35" s="7">
         <v>41731</v>
       </c>
-    </row>
-    <row r="37" spans="1:7">
+      <c r="C35" s="6"/>
+      <c r="D35" s="6"/>
+      <c r="E35" s="6"/>
+      <c r="F35" s="6"/>
+      <c r="G35" s="6"/>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="38" spans="1:7">
-      <c r="A38" s="1" t="s">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A38" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="B38" s="1">
+      <c r="B38" s="5">
         <v>0</v>
       </c>
-      <c r="C38" s="1">
+      <c r="C38" s="5">
         <v>1</v>
       </c>
-      <c r="D38" s="1">
+      <c r="D38" s="5">
         <v>2</v>
       </c>
-      <c r="E38" s="1">
+      <c r="E38" s="5">
         <v>3</v>
       </c>
-      <c r="F38" s="1">
+      <c r="F38" s="5">
         <v>4</v>
       </c>
-      <c r="G38" s="1">
+      <c r="G38" s="5">
         <v>5</v>
       </c>
     </row>
-    <row r="39" spans="1:7">
-      <c r="A39" t="s">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A39" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="B39" s="2">
+      <c r="B39" s="7">
         <v>-9475713</v>
       </c>
-      <c r="C39" s="2">
-        <v>1795856</v>
-      </c>
-      <c r="D39" s="2">
-        <v>1795856</v>
-      </c>
-      <c r="E39" s="2">
-        <v>1795856</v>
-      </c>
-      <c r="F39" s="2">
-        <v>1795856</v>
-      </c>
-      <c r="G39" s="2">
-        <v>1795856</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7">
-      <c r="A40" t="s">
+      <c r="C39" s="7">
+        <v>1542391</v>
+      </c>
+      <c r="D39" s="7">
+        <v>1542391</v>
+      </c>
+      <c r="E39" s="7">
+        <v>1542391</v>
+      </c>
+      <c r="F39" s="7">
+        <v>1542391</v>
+      </c>
+      <c r="G39" s="7">
+        <v>1542391</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A40" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="B40" s="3">
+      <c r="B40" s="8">
         <v>0.16</v>
       </c>
-    </row>
-    <row r="41" spans="1:7">
-      <c r="A41" t="s">
+      <c r="C40" s="6"/>
+      <c r="D40" s="6"/>
+      <c r="E40" s="6"/>
+      <c r="F40" s="6"/>
+      <c r="G40" s="6"/>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A41" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="B41" s="2">
+      <c r="B41" s="7">
         <f>NPV(B40,C39:G39)+B39</f>
-        <v>-3595554</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7">
-      <c r="A42" t="s">
+        <v>-4425471.9372357922</v>
+      </c>
+      <c r="C41" s="6"/>
+      <c r="D41" s="6"/>
+      <c r="E41" s="6"/>
+      <c r="F41" s="6"/>
+      <c r="G41" s="6"/>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A42" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B42" s="3">
+      <c r="B42" s="8">
         <f>IRR(B39:G39)</f>
-        <v>-0.017673467071406213</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7">
-      <c r="A43" t="s">
+        <v>-6.4946723735559542E-2</v>
+      </c>
+      <c r="C42" s="6"/>
+      <c r="D42" s="6"/>
+      <c r="E42" s="6"/>
+      <c r="F42" s="6"/>
+      <c r="G42" s="6"/>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A43" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="B43" s="2">
+      <c r="B43" s="7">
         <f>B39</f>
         <v>-9475713</v>
       </c>
-      <c r="C43" s="2">
+      <c r="C43" s="7">
         <f>B43+C39</f>
-        <v>-7679857</v>
-      </c>
-      <c r="D43" s="2">
+        <v>-7933322</v>
+      </c>
+      <c r="D43" s="7">
         <f>C43+D39</f>
-        <v>-5884002</v>
-      </c>
-      <c r="E43" s="2">
+        <v>-6390931</v>
+      </c>
+      <c r="E43" s="7">
         <f>D43+E39</f>
-        <v>-4088146</v>
-      </c>
-      <c r="F43" s="2">
+        <v>-4848540</v>
+      </c>
+      <c r="F43" s="7">
         <f>E43+F39</f>
-        <v>-2292290</v>
-      </c>
-      <c r="G43" s="2">
+        <v>-3306149</v>
+      </c>
+      <c r="G43" s="7">
         <f>F43+G39</f>
-        <v>-496434</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7">
-      <c r="A44" t="s">
+        <v>-1763758</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A44" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="B44" s="2">
+      <c r="B44" s="7">
         <f>B39</f>
         <v>-9475713</v>
       </c>
-      <c r="C44" s="2">
+      <c r="C44" s="7">
         <f>B44+C39/(1+B40)^1</f>
-        <v>-7927562</v>
-      </c>
-      <c r="D44" s="2">
+        <v>-8146065.5862068962</v>
+      </c>
+      <c r="D44" s="7">
         <f>C44+D39/(1+B40)^2</f>
-        <v>-6592948</v>
-      </c>
-      <c r="E44" s="2">
+        <v>-6999817.8156956006</v>
+      </c>
+      <c r="E44" s="7">
         <f>D44+E39/(1+B40)^3</f>
-        <v>-5442419</v>
-      </c>
-      <c r="F44" s="2">
+        <v>-6011673.1859444827</v>
+      </c>
+      <c r="F44" s="7">
         <f>E44+F39/(1+B40)^4</f>
-        <v>-4450584</v>
-      </c>
-      <c r="G44" s="2">
+        <v>-5159824.3671935191</v>
+      </c>
+      <c r="G44" s="7">
         <f>F44+G39/(1+B40)^5</f>
-        <v>-3595554</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7">
-      <c r="A45" t="s">
+        <v>-4425471.9372357922</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A45" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="B45" t="s">
+      <c r="B45" s="6" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="46" spans="1:7">
-      <c r="A46" t="s">
+      <c r="C45" s="6"/>
+      <c r="D45" s="6"/>
+      <c r="E45" s="6"/>
+      <c r="F45" s="6"/>
+      <c r="G45" s="6"/>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A46" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B46" s="2">
-        <v>103944</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7">
-      <c r="A47" t="s">
+      <c r="B46" s="7">
+        <v>91271</v>
+      </c>
+      <c r="C46" s="6"/>
+      <c r="D46" s="6"/>
+      <c r="E46" s="6"/>
+      <c r="F46" s="6"/>
+      <c r="G46" s="6"/>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A47" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="B47" s="2">
+      <c r="B47" s="7">
         <v>158850</v>
       </c>
-    </row>
-    <row r="49" spans="1:7">
+      <c r="C47" s="6"/>
+      <c r="D47" s="6"/>
+      <c r="E47" s="6"/>
+      <c r="F47" s="6"/>
+      <c r="G47" s="6"/>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="50" spans="1:7">
-      <c r="A50" s="1" t="s">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A50" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="B50" s="1">
+      <c r="B50" s="5">
         <v>0</v>
       </c>
-      <c r="C50" s="1">
+      <c r="C50" s="5">
         <v>1</v>
       </c>
-      <c r="D50" s="1">
+      <c r="D50" s="5">
         <v>2</v>
       </c>
-      <c r="E50" s="1">
+      <c r="E50" s="5">
         <v>3</v>
       </c>
-      <c r="F50" s="1">
+      <c r="F50" s="5">
         <v>4</v>
       </c>
-      <c r="G50" s="1">
+      <c r="G50" s="5">
         <v>5</v>
       </c>
     </row>
-    <row r="51" spans="1:7">
-      <c r="A51" t="s">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A51" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="B51" s="2">
+      <c r="B51" s="7">
         <v>-9475713</v>
       </c>
-      <c r="C51" s="2">
-        <v>5873167</v>
-      </c>
-      <c r="D51" s="2">
-        <v>5873167</v>
-      </c>
-      <c r="E51" s="2">
-        <v>5873167</v>
-      </c>
-      <c r="F51" s="2">
-        <v>5873167</v>
-      </c>
-      <c r="G51" s="2">
-        <v>7288309</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7">
-      <c r="A52" t="s">
+      <c r="C51" s="7">
+        <v>5366238</v>
+      </c>
+      <c r="D51" s="7">
+        <v>5366238</v>
+      </c>
+      <c r="E51" s="7">
+        <v>5366238</v>
+      </c>
+      <c r="F51" s="7">
+        <v>5366238</v>
+      </c>
+      <c r="G51" s="7">
+        <v>6781381</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A52" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="B52" s="3">
-        <v>0.1200564971751412</v>
-      </c>
-    </row>
-    <row r="53" spans="1:7">
-      <c r="A53" t="s">
+      <c r="B52" s="8">
+        <v>0.12005649717514121</v>
+      </c>
+      <c r="C52" s="6"/>
+      <c r="D52" s="6"/>
+      <c r="E52" s="6"/>
+      <c r="F52" s="6"/>
+      <c r="G52" s="6"/>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A53" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="B53" s="2">
+      <c r="B53" s="7">
         <f>NPV(B52,C51:G51)+B51</f>
-        <v>12495563</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7">
-      <c r="A54" t="s">
+        <v>10668454.563164886</v>
+      </c>
+      <c r="C53" s="6"/>
+      <c r="D53" s="6"/>
+      <c r="E53" s="6"/>
+      <c r="F53" s="6"/>
+      <c r="G53" s="6"/>
+    </row>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A54" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B54" s="3">
+      <c r="B54" s="8">
         <f>IRR(B51:G51)</f>
-        <v>0.5622259805332861</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7">
-      <c r="A55" t="s">
+        <v>0.50205327658958065</v>
+      </c>
+      <c r="C54" s="6"/>
+      <c r="D54" s="6"/>
+      <c r="E54" s="6"/>
+      <c r="F54" s="6"/>
+      <c r="G54" s="6"/>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A55" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="B55" s="2">
+      <c r="B55" s="7">
         <f>B51</f>
         <v>-9475713</v>
       </c>
-      <c r="C55" s="2">
+      <c r="C55" s="7">
         <f>B55+C51</f>
-        <v>-3602546</v>
-      </c>
-      <c r="D55" s="2">
+        <v>-4109475</v>
+      </c>
+      <c r="D55" s="7">
         <f>C55+D51</f>
-        <v>2270620</v>
-      </c>
-      <c r="E55" s="2">
+        <v>1256763</v>
+      </c>
+      <c r="E55" s="7">
         <f>D55+E51</f>
-        <v>8143787</v>
-      </c>
-      <c r="F55" s="2">
+        <v>6623001</v>
+      </c>
+      <c r="F55" s="7">
         <f>E55+F51</f>
-        <v>14016954</v>
-      </c>
-      <c r="G55" s="2">
+        <v>11989239</v>
+      </c>
+      <c r="G55" s="7">
         <f>F55+G51</f>
-        <v>21305263</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7">
-      <c r="A56" t="s">
+        <v>18770620</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A56" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="B56" s="2">
+      <c r="B56" s="7">
         <f>B51</f>
         <v>-9475713</v>
       </c>
-      <c r="C56" s="2">
+      <c r="C56" s="7">
         <f>B56+C51/(1+B52)^1</f>
-        <v>-4232079</v>
-      </c>
-      <c r="D56" s="2">
+        <v>-4684670.7503152583</v>
+      </c>
+      <c r="D56" s="7">
         <f>C56+D51/(1+B52)^2</f>
-        <v>449502</v>
-      </c>
-      <c r="E56" s="2">
+        <v>-407170.22978966311</v>
+      </c>
+      <c r="E56" s="7">
         <f>D56+E51/(1+B52)^3</f>
-        <v>4629273</v>
-      </c>
-      <c r="F56" s="2">
+        <v>3411834.0180440336</v>
+      </c>
+      <c r="F56" s="7">
         <f>E56+F51/(1+B52)^4</f>
-        <v>8361024</v>
-      </c>
-      <c r="G56" s="2">
+        <v>6821487.2430960611</v>
+      </c>
+      <c r="G56" s="7">
         <f>F56+G51/(1+B52)^5</f>
-        <v>12495563</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7">
-      <c r="A57" t="s">
+        <v>10668454.56316489</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A57" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="B57" t="s">
+      <c r="B57" s="6" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="58" spans="1:7">
-      <c r="A58" t="s">
+      <c r="C57" s="6"/>
+      <c r="D57" s="6"/>
+      <c r="E57" s="6"/>
+      <c r="F57" s="6"/>
+      <c r="G57" s="6"/>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A58" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B58" s="2">
-        <v>152136</v>
-      </c>
-    </row>
-    <row r="59" spans="1:7">
-      <c r="A59" t="s">
+      <c r="B58" s="7">
+        <v>139463</v>
+      </c>
+      <c r="C58" s="6"/>
+      <c r="D58" s="6"/>
+      <c r="E58" s="6"/>
+      <c r="F58" s="6"/>
+      <c r="G58" s="6"/>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A59" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="B59" s="2">
+      <c r="B59" s="7">
         <v>65464</v>
       </c>
-    </row>
-    <row r="61" spans="1:7">
+      <c r="C59" s="6"/>
+      <c r="D59" s="6"/>
+      <c r="E59" s="6"/>
+      <c r="F59" s="6"/>
+      <c r="G59" s="6"/>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A61" s="1" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="62" spans="1:7">
-      <c r="A62" s="1" t="s">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A62" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="B62" s="1">
+      <c r="B62" s="5">
         <v>0</v>
       </c>
-      <c r="C62" s="1">
+      <c r="C62" s="5">
         <v>1</v>
       </c>
-      <c r="D62" s="1">
+      <c r="D62" s="5">
         <v>2</v>
       </c>
-      <c r="E62" s="1">
+      <c r="E62" s="5">
         <v>3</v>
       </c>
-      <c r="F62" s="1">
+      <c r="F62" s="5">
         <v>4</v>
       </c>
-      <c r="G62" s="1">
+      <c r="G62" s="5">
         <v>5</v>
       </c>
     </row>
-    <row r="63" spans="1:7">
-      <c r="A63" t="s">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A63" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="B63" s="2">
+      <c r="B63" s="7">
         <v>-9475713</v>
       </c>
-      <c r="C63" s="2">
-        <v>11083277</v>
-      </c>
-      <c r="D63" s="2">
-        <v>11083277</v>
-      </c>
-      <c r="E63" s="2">
-        <v>11083277</v>
-      </c>
-      <c r="F63" s="2">
-        <v>11083277</v>
-      </c>
-      <c r="G63" s="2">
-        <v>13913562</v>
-      </c>
-    </row>
-    <row r="64" spans="1:7">
-      <c r="A64" t="s">
+      <c r="C63" s="7">
+        <v>10322884</v>
+      </c>
+      <c r="D63" s="7">
+        <v>10322884</v>
+      </c>
+      <c r="E63" s="7">
+        <v>10322884</v>
+      </c>
+      <c r="F63" s="7">
+        <v>10322884</v>
+      </c>
+      <c r="G63" s="7">
+        <v>13153169</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A64" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="B64" s="3">
+      <c r="B64" s="8">
         <v>0.08</v>
       </c>
-    </row>
-    <row r="65" spans="1:7">
-      <c r="A65" t="s">
+      <c r="C64" s="6"/>
+      <c r="D64" s="6"/>
+      <c r="E64" s="6"/>
+      <c r="F64" s="6"/>
+      <c r="G64" s="6"/>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A65" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="B65" s="2">
+      <c r="B65" s="7">
         <f>NPV(B64,C63:G63)+B63</f>
-        <v>36702841</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7">
-      <c r="A66" t="s">
+        <v>33666813.972209439</v>
+      </c>
+      <c r="C65" s="6"/>
+      <c r="D65" s="6"/>
+      <c r="E65" s="6"/>
+      <c r="F65" s="6"/>
+      <c r="G65" s="6"/>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A66" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="B66" s="3">
+      <c r="B66" s="8">
         <f>IRR(B63:G63)</f>
-        <v>1.1517519873775988</v>
-      </c>
-    </row>
-    <row r="67" spans="1:7">
-      <c r="A67" t="s">
+        <v>1.069098256100371</v>
+      </c>
+      <c r="C66" s="6"/>
+      <c r="D66" s="6"/>
+      <c r="E66" s="6"/>
+      <c r="F66" s="6"/>
+      <c r="G66" s="6"/>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A67" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="B67" s="2">
+      <c r="B67" s="7">
         <f>B63</f>
         <v>-9475713</v>
       </c>
-      <c r="C67" s="2">
+      <c r="C67" s="7">
         <f>B67+C63</f>
-        <v>1607564</v>
-      </c>
-      <c r="D67" s="2">
+        <v>847171</v>
+      </c>
+      <c r="D67" s="7">
         <f>C67+D63</f>
-        <v>12690840</v>
-      </c>
-      <c r="E67" s="2">
+        <v>11170055</v>
+      </c>
+      <c r="E67" s="7">
         <f>D67+E63</f>
-        <v>23774117</v>
-      </c>
-      <c r="F67" s="2">
+        <v>21492939</v>
+      </c>
+      <c r="F67" s="7">
         <f>E67+F63</f>
-        <v>34857393</v>
-      </c>
-      <c r="G67" s="2">
+        <v>31815823</v>
+      </c>
+      <c r="G67" s="7">
         <f>F67+G63</f>
-        <v>48770955</v>
-      </c>
-    </row>
-    <row r="68" spans="1:7">
-      <c r="A68" t="s">
+        <v>44968992</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A68" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="B68" s="2">
+      <c r="B68" s="7">
         <f>B63</f>
         <v>-9475713</v>
       </c>
-      <c r="C68" s="2">
+      <c r="C68" s="7">
         <f>B68+C63/(1+B64)^1</f>
-        <v>786580</v>
-      </c>
-      <c r="D68" s="2">
+        <v>82512.925925925374</v>
+      </c>
+      <c r="D68" s="7">
         <f>C68+D63/(1+B64)^2</f>
-        <v>10288703</v>
-      </c>
-      <c r="E68" s="2">
+        <v>8932722.116598079</v>
+      </c>
+      <c r="E68" s="7">
         <f>D68+E63/(1+B64)^3</f>
-        <v>19086966</v>
-      </c>
-      <c r="F68" s="2">
+        <v>17127360.256109331</v>
+      </c>
+      <c r="F68" s="7">
         <f>E68+F63/(1+B64)^4</f>
-        <v>27233505</v>
-      </c>
-      <c r="G68" s="2">
+        <v>24714988.163064193</v>
+      </c>
+      <c r="G68" s="7">
         <f>F68+G63/(1+B64)^5</f>
-        <v>36702841</v>
-      </c>
-    </row>
-    <row r="69" spans="1:7">
-      <c r="A69" t="s">
+        <v>33666813.972209446</v>
+      </c>
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A69" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="B69" t="s">
+      <c r="B69" s="6" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="70" spans="1:7">
-      <c r="A70" t="s">
+      <c r="C69" s="6"/>
+      <c r="D69" s="6"/>
+      <c r="E69" s="6"/>
+      <c r="F69" s="6"/>
+      <c r="G69" s="6"/>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A70" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B70" s="2">
-        <v>187080</v>
-      </c>
-    </row>
-    <row r="71" spans="1:7">
-      <c r="A71" t="s">
+      <c r="B70" s="7">
+        <v>174407</v>
+      </c>
+      <c r="C70" s="6"/>
+      <c r="D70" s="6"/>
+      <c r="E70" s="6"/>
+      <c r="F70" s="6"/>
+      <c r="G70" s="6"/>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A71" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="B71" s="2">
+      <c r="B71" s="7">
         <v>33872</v>
       </c>
+      <c r="C71" s="6"/>
+      <c r="D71" s="6"/>
+      <c r="E71" s="6"/>
+      <c r="F71" s="6"/>
+      <c r="G71" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2495,293 +2746,298 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D30"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:D31"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.7109375" customWidth="1"/>
-    <col min="2" max="2" width="95.7109375" customWidth="1"/>
-    <col min="3" max="4" width="14.7109375" customWidth="1"/>
+    <col min="1" max="1" width="22.6640625" customWidth="1"/>
+    <col min="2" max="2" width="95.6640625" customWidth="1"/>
+    <col min="3" max="4" width="14.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="5" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
-      <c r="A2" t="s">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" s="7">
         <v>4124213</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="6" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
-      <c r="A3" t="s">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="7">
         <v>250634</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="6" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
-      <c r="A4" t="s">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="7">
         <v>802156</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="6" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
-      <c r="A5" t="s">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5" s="7">
         <v>1188042</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="6" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
-      <c r="A6" t="s">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6" s="7">
         <v>3248117</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="6" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
-      <c r="A7" t="s">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="C7" s="2">
+      <c r="C7" s="7">
         <v>1117016</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="6" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
-      <c r="A8" t="s">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="C8" s="2">
+      <c r="C8" s="7">
         <v>1203712</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="6" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
-      <c r="A9" t="s">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="C9" s="2">
+      <c r="C9" s="7">
         <v>2400000</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="6" t="s">
         <v>111</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
-      <c r="A10" t="s">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="C10" s="2">
+      <c r="C10" s="7">
         <v>2494370</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="6" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="11" spans="1:4">
-      <c r="B11" s="1" t="s">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B11" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="C11" s="2">
+      <c r="C11" s="7">
         <f>SUMIF(D2:D10,"A",C2:C10)</f>
         <v>14333890</v>
       </c>
     </row>
-    <row r="12" spans="1:4">
-      <c r="B12" s="1" t="s">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B12" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="C12" s="2">
+      <c r="C12" s="7">
         <f>C11+SUMIF(D2:D10,"B",C2:C10)</f>
         <v>16828260</v>
       </c>
     </row>
-    <row r="13" spans="1:4">
-      <c r="B13" s="1" t="s">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B13" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="C13" s="2">
+      <c r="C13" s="7">
         <v>7352547</v>
       </c>
     </row>
-    <row r="14" spans="1:4">
-      <c r="B14" s="1" t="s">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B14" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="C14" s="2">
+      <c r="C14" s="7">
         <f>C12-C13</f>
         <v>9475713</v>
       </c>
     </row>
-    <row r="15" spans="1:4">
-      <c r="A15" t="s">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B15" s="3"/>
+      <c r="C15" s="4"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B16" s="10" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="16" spans="1:4">
-      <c r="B16" t="s">
+    <row r="17" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B17" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="C16">
-        <v>6.13</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4">
-      <c r="B17" t="s">
+      <c r="C17" s="6">
+        <v>5.13</v>
+      </c>
+    </row>
+    <row r="18" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B18" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="C17">
-        <v>9.300000000000001</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4">
-      <c r="B18" t="s">
+      <c r="C18" s="6">
+        <v>8.3000000000000007</v>
+      </c>
+    </row>
+    <row r="19" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B19" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="C18">
-        <v>12.47</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4">
-      <c r="B19" s="1" t="s">
+      <c r="C19" s="6">
+        <v>11.47</v>
+      </c>
+    </row>
+    <row r="20" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B20" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="C19" s="2">
+      <c r="C20" s="7">
         <v>2526946</v>
       </c>
-      <c r="D19" s="2">
+      <c r="D20" s="7">
         <v>11806944</v>
       </c>
     </row>
-    <row r="20" spans="1:4">
-      <c r="A20" t="s">
+    <row r="21" spans="2:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B21" s="11" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="23" spans="1:4">
-      <c r="A23" s="1" t="s">
+    <row r="24" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B24" s="5" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="24" spans="1:4">
-      <c r="B24" t="s">
+      <c r="C24" s="6"/>
+    </row>
+    <row r="25" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B25" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="C24" s="2">
+      <c r="C25" s="7">
         <v>2494370</v>
       </c>
     </row>
-    <row r="25" spans="1:4">
-      <c r="B25" t="s">
+    <row r="26" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B26" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="C25" s="2">
+      <c r="C26" s="7">
         <v>1014882</v>
       </c>
     </row>
-    <row r="26" spans="1:4">
-      <c r="B26" t="s">
+    <row r="27" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B27" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="C26" s="2">
+      <c r="C27" s="7">
         <v>2331231</v>
       </c>
     </row>
-    <row r="27" spans="1:4">
-      <c r="B27" t="s">
+    <row r="28" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B28" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="C27" s="2">
+      <c r="C28" s="7">
         <v>52000</v>
       </c>
     </row>
-    <row r="28" spans="1:4">
-      <c r="B28" t="s">
+    <row r="29" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B29" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="C28" s="2">
+      <c r="C29" s="7">
         <v>100652</v>
       </c>
     </row>
-    <row r="29" spans="1:4">
-      <c r="B29" t="s">
+    <row r="30" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B30" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="C29" s="2">
+      <c r="C30" s="7">
         <v>1203712</v>
       </c>
     </row>
-    <row r="30" spans="1:4">
-      <c r="B30" t="s">
+    <row r="31" spans="2:4" x14ac:dyDescent="0.3">
+      <c r="B31" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="C30" s="2">
+      <c r="C31" s="7">
         <v>155700</v>
       </c>
     </row>
@@ -2791,132 +3047,132 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:I6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.7109375" customWidth="1"/>
-    <col min="2" max="11" width="14.7109375" customWidth="1"/>
+    <col min="1" max="1" width="16.6640625" customWidth="1"/>
+    <col min="2" max="11" width="14.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="F3" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="G3" s="5" t="s">
         <v>152</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="H3" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="I3" s="5" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
-      <c r="A4" t="s">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A4" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="6">
         <v>20</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="7">
         <v>-80684</v>
       </c>
-      <c r="D4" s="3">
+      <c r="D4" s="8">
         <v>0.16</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="7">
         <v>-24001624</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="G4" s="2">
+      <c r="G4" s="7">
         <v>-16828260</v>
       </c>
-      <c r="H4" s="2">
+      <c r="H4" s="7">
         <v>-2190813</v>
       </c>
-      <c r="I4" s="2">
+      <c r="I4" s="7">
         <v>-2190813</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
-      <c r="A5" t="s">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="6">
         <v>40</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5" s="7">
         <v>-29991</v>
       </c>
-      <c r="D5" s="3">
-        <v>0.1200564971751412</v>
-      </c>
-      <c r="E5" s="2">
+      <c r="D5" s="8">
+        <v>0.12005649717514121</v>
+      </c>
+      <c r="E5" s="7">
         <v>-21075242</v>
       </c>
-      <c r="F5" s="3">
-        <v>-0.5967910214694709</v>
-      </c>
-      <c r="G5" s="2">
+      <c r="F5" s="8">
+        <v>-0.59679102146947094</v>
+      </c>
+      <c r="G5" s="7">
         <v>-16828260</v>
       </c>
-      <c r="H5" s="2">
+      <c r="H5" s="7">
         <v>-1632498</v>
       </c>
-      <c r="I5" s="2">
+      <c r="I5" s="7">
         <v>1253154</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
-      <c r="A6" t="s">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="6">
         <v>60</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6" s="7">
         <v>7543</v>
       </c>
-      <c r="D6" s="3">
+      <c r="D6" s="8">
         <v>0.08</v>
       </c>
-      <c r="E6" s="2">
+      <c r="E6" s="7">
         <v>-12245648</v>
       </c>
-      <c r="F6" s="3">
-        <v>-0.1771573409565363</v>
-      </c>
-      <c r="G6" s="2">
+      <c r="F6" s="8">
+        <v>-0.17715734095653629</v>
+      </c>
+      <c r="G6" s="7">
         <v>-16828260</v>
       </c>
-      <c r="H6" s="2">
+      <c r="H6" s="7">
         <v>163989</v>
       </c>
-      <c r="I6" s="2">
+      <c r="I6" s="7">
         <v>5935293</v>
       </c>
     </row>
@@ -2926,189 +3182,189 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:G10"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="40.7109375" customWidth="1"/>
-    <col min="2" max="7" width="14.7109375" customWidth="1"/>
+    <col min="1" max="1" width="40.6640625" customWidth="1"/>
+    <col min="2" max="7" width="14.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
-      <c r="A1" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="B1">
+      <c r="B1" s="6">
         <v>22.99836354166813</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
-      <c r="A2" t="s">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
         <v>157</v>
       </c>
-      <c r="B2">
-        <v>13.28711111111036</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
-      <c r="A4" s="1" t="s">
+      <c r="B2" s="6">
+        <v>13.287111111110359</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="5" t="s">
         <v>158</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="F4" s="5" t="s">
         <v>162</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="G4" s="5" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
-      <c r="A5" s="2">
-        <v>1144.3472</v>
-      </c>
-      <c r="B5" s="2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="7">
+        <v>1144.3471999999999</v>
+      </c>
+      <c r="B5" s="7">
         <v>26318.11292349</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5" s="7">
         <v>20</v>
       </c>
-      <c r="D5" s="2">
-        <v>526362.2584698001</v>
-      </c>
-      <c r="E5" s="2">
-        <v>2101611.87253146</v>
-      </c>
-      <c r="F5" s="2">
+      <c r="D5" s="7">
+        <v>526362.25846980012</v>
+      </c>
+      <c r="E5" s="7">
+        <v>2101611.8725314601</v>
+      </c>
+      <c r="F5" s="7">
         <v>1897152.607900783</v>
       </c>
-      <c r="G5" s="2">
-        <v>1723464.602434462</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
-      <c r="A6" s="2">
-        <v>1144.3472</v>
-      </c>
-      <c r="B6" s="2">
+      <c r="G5" s="7">
+        <v>1723464.6024344619</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" s="7">
+        <v>1144.3471999999999</v>
+      </c>
+      <c r="B6" s="7">
         <v>26318.11292349</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6" s="7">
         <v>40</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="7">
         <v>1052724.5169396</v>
       </c>
-      <c r="E6" s="2">
-        <v>4203223.74506292</v>
-      </c>
-      <c r="F6" s="2">
-        <v>3794305.215801567</v>
-      </c>
-      <c r="G6" s="2">
-        <v>3446929.204868924</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
-      <c r="A7" s="2">
-        <v>1144.3472</v>
-      </c>
-      <c r="B7" s="2">
+      <c r="E6" s="7">
+        <v>4203223.7450629203</v>
+      </c>
+      <c r="F6" s="7">
+        <v>3794305.2158015668</v>
+      </c>
+      <c r="G6" s="7">
+        <v>3446929.2048689239</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" s="7">
+        <v>1144.3471999999999</v>
+      </c>
+      <c r="B7" s="7">
         <v>26318.11292349</v>
       </c>
-      <c r="C7" s="2">
+      <c r="C7" s="7">
         <v>60</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D7" s="7">
         <v>1579086.7754094</v>
       </c>
-      <c r="E7" s="2">
-        <v>6304835.61759438</v>
-      </c>
-      <c r="F7" s="2">
-        <v>5691457.82370235</v>
-      </c>
-      <c r="G7" s="2">
-        <v>5170393.807303385</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7">
-      <c r="A8" s="2">
-        <v>953.6227</v>
-      </c>
-      <c r="B8" s="2">
-        <v>21931.76153618712</v>
-      </c>
-      <c r="C8" s="2">
+      <c r="E7" s="7">
+        <v>6304835.6175943799</v>
+      </c>
+      <c r="F7" s="7">
+        <v>5691457.8237023503</v>
+      </c>
+      <c r="G7" s="7">
+        <v>5170393.8073033849</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" s="7">
+        <v>953.62270000000001</v>
+      </c>
+      <c r="B8" s="7">
+        <v>21931.761536187121</v>
+      </c>
+      <c r="C8" s="7">
         <v>20</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="7">
         <v>438635.2307237424</v>
       </c>
-      <c r="E8" s="2">
-        <v>1751343.288326748</v>
-      </c>
-      <c r="F8" s="2">
+      <c r="E8" s="7">
+        <v>1751343.2883267479</v>
+      </c>
+      <c r="F8" s="7">
         <v>1580960.561845554</v>
       </c>
-      <c r="G8" s="2">
-        <v>1436220.552230982</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7">
-      <c r="A9" s="2">
-        <v>953.6227</v>
-      </c>
-      <c r="B9" s="2">
-        <v>21931.76153618712</v>
-      </c>
-      <c r="C9" s="2">
+      <c r="G8" s="7">
+        <v>1436220.5522309821</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="7">
+        <v>953.62270000000001</v>
+      </c>
+      <c r="B9" s="7">
+        <v>21931.761536187121</v>
+      </c>
+      <c r="C9" s="7">
         <v>40</v>
       </c>
-      <c r="D9" s="2">
-        <v>877270.4614474848</v>
-      </c>
-      <c r="E9" s="2">
+      <c r="D9" s="7">
+        <v>877270.46144748479</v>
+      </c>
+      <c r="E9" s="7">
         <v>3502686.576653495</v>
       </c>
-      <c r="F9" s="2">
-        <v>3161921.123691107</v>
-      </c>
-      <c r="G9" s="2">
-        <v>2872441.104461964</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7">
-      <c r="A10" s="2">
-        <v>953.6227</v>
-      </c>
-      <c r="B10" s="2">
-        <v>21931.76153618712</v>
-      </c>
-      <c r="C10" s="2">
+      <c r="F9" s="7">
+        <v>3161921.1236911071</v>
+      </c>
+      <c r="G9" s="7">
+        <v>2872441.1044619642</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" s="7">
+        <v>953.62270000000001</v>
+      </c>
+      <c r="B10" s="7">
+        <v>21931.761536187121</v>
+      </c>
+      <c r="C10" s="7">
         <v>60</v>
       </c>
-      <c r="D10" s="2">
+      <c r="D10" s="7">
         <v>1315905.692171227</v>
       </c>
-      <c r="E10" s="2">
-        <v>5254029.864980243</v>
-      </c>
-      <c r="F10" s="2">
-        <v>4742881.685536661</v>
-      </c>
-      <c r="G10" s="2">
-        <v>4308661.656692945</v>
+      <c r="E10" s="7">
+        <v>5254029.8649802431</v>
+      </c>
+      <c r="F10" s="7">
+        <v>4742881.6855366612</v>
+      </c>
+      <c r="G10" s="7">
+        <v>4308661.6566929454</v>
       </c>
     </row>
   </sheetData>
@@ -3117,147 +3373,147 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:D14"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.7109375" customWidth="1"/>
-    <col min="2" max="2" width="62.7109375" customWidth="1"/>
-    <col min="3" max="3" width="10.7109375" customWidth="1"/>
-    <col min="4" max="4" width="48.7109375" customWidth="1"/>
+    <col min="1" max="1" width="18.6640625" customWidth="1"/>
+    <col min="2" max="2" width="62.6640625" customWidth="1"/>
+    <col min="3" max="3" width="10.6640625" customWidth="1"/>
+    <col min="4" max="4" width="48.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="s">
         <v>165</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="5" t="s">
         <v>166</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="5" t="s">
         <v>167</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="5" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
-      <c r="A4" t="s">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="6">
         <v>3</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="6" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="5" spans="1:4">
-      <c r="A5" t="s">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="s">
         <v>172</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="6" t="s">
         <v>173</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="6">
         <v>3</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="6" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
-      <c r="A6" t="s">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="6">
         <v>3</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="6" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
-      <c r="A7" t="s">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="6" t="s">
         <v>179</v>
       </c>
-      <c r="C7">
+      <c r="C7" s="6">
         <v>3</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="6" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
-      <c r="A8" t="s">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
         <v>181</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="6" t="s">
         <v>182</v>
       </c>
-      <c r="C8">
+      <c r="C8" s="6">
         <v>3</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="6" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
-      <c r="A9" t="s">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="6" t="s">
         <v>184</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="6">
         <v>1</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="6" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
-      <c r="B10" s="1" t="s">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B10" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="6">
         <f>SUM(C4:C9)</f>
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="1:4">
-      <c r="B11" t="s">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B11" s="6" t="s">
         <v>188</v>
       </c>
-      <c r="C11" s="2">
+      <c r="C11" s="7">
         <v>100000</v>
       </c>
     </row>
-    <row r="12" spans="1:4">
-      <c r="B12" s="1" t="s">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B12" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="C12" s="2">
+      <c r="C12" s="7">
         <f>C10*C11</f>
         <v>1600000</v>
       </c>
     </row>
-    <row r="14" spans="1:4">
-      <c r="A14" s="4" t="s">
+    <row r="14" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="B14" s="2" t="s">
         <v>190</v>
       </c>
     </row>

</xml_diff>